<commit_message>
Pulmon de Oriente: integra 2026 (Seguridad+Movilidad+Cohesion) sin tocar linea base
- PATHS a listas [base, ext 2026]; load_gj concatena; procesar() hace coalesce fecha_hech/fecha_hecho
- Linea base 2023-2025 intacta; extensiones 2026 Q2-Q3 integradas (patron Barrio Obrero)
- FIX filtro riñas: contains('RI') (inflaba, capturaba INTEGRIDAD) -> == 'RIÑAS' exacto
  Linea base real riñas: 224/294/599 (antes 3362/3565/4310 por el bug)
- Anualiza 2026 parcial (x4/trim): seg/cohesion x1.33, siniestros x2 (como Roosevelt)
- Movilidad integrada (siniestros base+ext); umbrales recalibrados al rango real + 2026 anualizado
- ITT: 2023=47.9, 2024=56.8, 2025=48.3, 2026=26.6. Excel 7 hojas (+Movilidad)
- Pendiente integrar: EU/vivienda, DesEco, Educacion (datos ya cargados)
</commit_message>
<xml_diff>
--- a/outputs/itt_pulmon_oriente/ITT_Pulmon_Oriente_Consolidado.xlsx
+++ b/outputs/itt_pulmon_oriente/ITT_Pulmon_Oriente_Consolidado.xlsx
@@ -9,10 +9,11 @@
   <sheets>
     <sheet name="ITT_Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Seguridad" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cohesion_Social" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Indicadores_Trimestrales" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Dimensiones_Pendientes" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Metadatos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Movilidad" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cohesion_Social" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Indicadores_Trimestrales" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dimensiones_Pendientes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Metadatos" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +441,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
     <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -496,20 +497,22 @@
         <v>2023</v>
       </c>
       <c r="B2" t="n">
-        <v>24.03</v>
-      </c>
-      <c r="C2" t="inlineStr"/>
+        <v>39.98</v>
+      </c>
+      <c r="C2" t="n">
+        <v>34.21</v>
+      </c>
       <c r="D2" t="n">
-        <v>57.43</v>
+        <v>75.14</v>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>37.8</v>
+        <v>47.9</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Activacion</t>
+          <t>Consolidacion</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -523,16 +526,18 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>37.89</v>
-      </c>
-      <c r="C3" t="inlineStr"/>
+        <v>52.71</v>
+      </c>
+      <c r="C3" t="n">
+        <v>46.85</v>
+      </c>
       <c r="D3" t="n">
-        <v>57.28</v>
+        <v>73.98999999999999</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>45.9</v>
+        <v>56.8</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -550,16 +555,18 @@
         <v>2025</v>
       </c>
       <c r="B4" t="n">
-        <v>54.39</v>
-      </c>
-      <c r="C4" t="inlineStr"/>
+        <v>61.51</v>
+      </c>
+      <c r="C4" t="n">
+        <v>33.62</v>
+      </c>
       <c r="D4" t="n">
-        <v>27.9</v>
+        <v>46.52</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>43.5</v>
+        <v>48.3</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -577,20 +584,22 @@
         <v>2026</v>
       </c>
       <c r="B5" t="n">
-        <v>74.45999999999999</v>
-      </c>
-      <c r="C5" t="inlineStr"/>
+        <v>26.67</v>
+      </c>
+      <c r="C5" t="n">
+        <v>37.38</v>
+      </c>
       <c r="D5" t="n">
-        <v>76.95999999999999</v>
+        <v>13.94</v>
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>75.5</v>
+        <v>26.6</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Transformacion</t>
+          <t>Activacion</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -667,10 +676,10 @@
         <v>16.43</v>
       </c>
       <c r="E2" t="n">
-        <v>31.62</v>
+        <v>63.53</v>
       </c>
       <c r="F2" t="n">
-        <v>24.03</v>
+        <v>39.98</v>
       </c>
     </row>
     <row r="3">
@@ -687,10 +696,10 @@
         <v>39.29</v>
       </c>
       <c r="E3" t="n">
-        <v>36.5</v>
+        <v>66.13</v>
       </c>
       <c r="F3" t="n">
-        <v>37.89</v>
+        <v>52.71</v>
       </c>
     </row>
     <row r="4">
@@ -707,10 +716,10 @@
         <v>39.29</v>
       </c>
       <c r="E4" t="n">
-        <v>69.5</v>
+        <v>83.73</v>
       </c>
       <c r="F4" t="n">
-        <v>54.39</v>
+        <v>61.51</v>
       </c>
     </row>
     <row r="5">
@@ -718,19 +727,19 @@
         <v>2026</v>
       </c>
       <c r="B5" t="n">
-        <v>26</v>
+        <v>91</v>
       </c>
       <c r="C5" t="n">
-        <v>1160</v>
+        <v>2125</v>
       </c>
       <c r="D5" t="n">
-        <v>81.43000000000001</v>
+        <v>35</v>
       </c>
       <c r="E5" t="n">
-        <v>67.5</v>
+        <v>18.33</v>
       </c>
       <c r="F5" t="n">
-        <v>74.45999999999999</v>
+        <v>26.67</v>
       </c>
     </row>
   </sheetData>
@@ -739,6 +748,176 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>año</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>siniestralidad</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>lesionados</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>mortales</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>score_siniestralidad</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>score_lesionados</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>score_mortales</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>score_movilidad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B2" t="n">
+        <v>236</v>
+      </c>
+      <c r="C2" t="n">
+        <v>194</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18</v>
+      </c>
+      <c r="E2" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>47.14</v>
+      </c>
+      <c r="G2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H2" t="n">
+        <v>34.21</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="n">
+        <v>222</v>
+      </c>
+      <c r="C3" t="n">
+        <v>198</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3" t="n">
+        <v>36.25</v>
+      </c>
+      <c r="F3" t="n">
+        <v>44.29</v>
+      </c>
+      <c r="G3" t="n">
+        <v>60</v>
+      </c>
+      <c r="H3" t="n">
+        <v>46.85</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" t="n">
+        <v>229</v>
+      </c>
+      <c r="C4" t="n">
+        <v>197</v>
+      </c>
+      <c r="D4" t="n">
+        <v>19</v>
+      </c>
+      <c r="E4" t="n">
+        <v>31.88</v>
+      </c>
+      <c r="F4" t="n">
+        <v>45</v>
+      </c>
+      <c r="G4" t="n">
+        <v>24</v>
+      </c>
+      <c r="H4" t="n">
+        <v>33.62</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="n">
+        <v>240</v>
+      </c>
+      <c r="C5" t="n">
+        <v>222</v>
+      </c>
+      <c r="D5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E5" t="n">
+        <v>25</v>
+      </c>
+      <c r="F5" t="n">
+        <v>27.14</v>
+      </c>
+      <c r="G5" t="n">
+        <v>60</v>
+      </c>
+      <c r="H5" t="n">
+        <v>37.38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -807,22 +986,22 @@
         <v>482</v>
       </c>
       <c r="C2" t="n">
-        <v>3362</v>
+        <v>224</v>
       </c>
       <c r="D2" t="n">
         <v>859</v>
       </c>
       <c r="E2" t="n">
-        <v>63.6</v>
+        <v>74</v>
       </c>
       <c r="F2" t="n">
-        <v>54.6</v>
+        <v>85.41</v>
       </c>
       <c r="G2" t="n">
-        <v>54.1</v>
+        <v>66</v>
       </c>
       <c r="H2" t="n">
-        <v>57.43</v>
+        <v>75.14</v>
       </c>
     </row>
     <row r="3">
@@ -833,22 +1012,22 @@
         <v>520</v>
       </c>
       <c r="C3" t="n">
-        <v>3562</v>
+        <v>294</v>
       </c>
       <c r="D3" t="n">
         <v>721</v>
       </c>
       <c r="E3" t="n">
-        <v>56</v>
+        <v>68.56999999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>47.93</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>67.90000000000001</v>
+        <v>76.22</v>
       </c>
       <c r="H3" t="n">
-        <v>57.28</v>
+        <v>73.98999999999999</v>
       </c>
     </row>
     <row r="4">
@@ -859,22 +1038,22 @@
         <v>587</v>
       </c>
       <c r="C4" t="n">
-        <v>4307</v>
+        <v>599</v>
       </c>
       <c r="D4" t="n">
         <v>1220</v>
       </c>
       <c r="E4" t="n">
-        <v>42.6</v>
+        <v>59</v>
       </c>
       <c r="F4" t="n">
-        <v>23.1</v>
+        <v>41.29</v>
       </c>
       <c r="G4" t="n">
-        <v>18</v>
+        <v>39.26</v>
       </c>
       <c r="H4" t="n">
-        <v>27.9</v>
+        <v>46.52</v>
       </c>
     </row>
     <row r="5">
@@ -882,25 +1061,25 @@
         <v>2026</v>
       </c>
       <c r="B5" t="n">
-        <v>468</v>
+        <v>901</v>
       </c>
       <c r="C5" t="n">
-        <v>2382</v>
+        <v>825</v>
       </c>
       <c r="D5" t="n">
-        <v>628</v>
+        <v>1575</v>
       </c>
       <c r="E5" t="n">
-        <v>66.40000000000001</v>
+        <v>14.14</v>
       </c>
       <c r="F5" t="n">
-        <v>87.27</v>
+        <v>14.71</v>
       </c>
       <c r="G5" t="n">
-        <v>77.2</v>
+        <v>12.96</v>
       </c>
       <c r="H5" t="n">
-        <v>76.95999999999999</v>
+        <v>13.94</v>
       </c>
     </row>
   </sheetData>
@@ -908,7 +1087,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -925,7 +1104,7 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
     <col width="7" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
   </cols>
@@ -1001,19 +1180,19 @@
         <v>432</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H2" t="n">
         <v>115</v>
       </c>
       <c r="I2" t="n">
-        <v>658</v>
+        <v>70</v>
       </c>
       <c r="J2" t="n">
         <v>238</v>
@@ -1038,19 +1217,19 @@
         <v>375</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H3" t="n">
         <v>148</v>
       </c>
       <c r="I3" t="n">
-        <v>824</v>
+        <v>67</v>
       </c>
       <c r="J3" t="n">
         <v>222</v>
@@ -1075,19 +1254,19 @@
         <v>379</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
         <v>129</v>
       </c>
       <c r="I4" t="n">
-        <v>823</v>
+        <v>50</v>
       </c>
       <c r="J4" t="n">
         <v>222</v>
@@ -1112,19 +1291,19 @@
         <v>261</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H5" t="n">
         <v>90</v>
       </c>
       <c r="I5" t="n">
-        <v>1057</v>
+        <v>37</v>
       </c>
       <c r="J5" t="n">
         <v>177</v>
@@ -1149,19 +1328,19 @@
         <v>377</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H6" t="n">
         <v>108</v>
       </c>
       <c r="I6" t="n">
-        <v>1022</v>
+        <v>86</v>
       </c>
       <c r="J6" t="n">
         <v>136</v>
@@ -1186,19 +1365,19 @@
         <v>354</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
         <v>133</v>
       </c>
       <c r="I7" t="n">
-        <v>983</v>
+        <v>91</v>
       </c>
       <c r="J7" t="n">
         <v>270</v>
@@ -1223,19 +1402,19 @@
         <v>349</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H8" t="n">
         <v>141</v>
       </c>
       <c r="I8" t="n">
-        <v>625</v>
+        <v>55</v>
       </c>
       <c r="J8" t="n">
         <v>139</v>
@@ -1260,19 +1439,19 @@
         <v>328</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H9" t="n">
         <v>138</v>
       </c>
       <c r="I9" t="n">
-        <v>932</v>
+        <v>62</v>
       </c>
       <c r="J9" t="n">
         <v>176</v>
@@ -1297,19 +1476,19 @@
         <v>288</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H10" t="n">
         <v>128</v>
       </c>
       <c r="I10" t="n">
-        <v>1094</v>
+        <v>92</v>
       </c>
       <c r="J10" t="n">
         <v>239</v>
@@ -1334,19 +1513,19 @@
         <v>306</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H11" t="n">
         <v>149</v>
       </c>
       <c r="I11" t="n">
-        <v>948</v>
+        <v>120</v>
       </c>
       <c r="J11" t="n">
         <v>264</v>
@@ -1371,19 +1550,19 @@
         <v>291</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
         <v>199</v>
       </c>
       <c r="I12" t="n">
-        <v>895</v>
+        <v>144</v>
       </c>
       <c r="J12" t="n">
         <v>358</v>
@@ -1408,19 +1587,19 @@
         <v>259</v>
       </c>
       <c r="E13" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="H13" t="n">
         <v>111</v>
       </c>
       <c r="I13" t="n">
-        <v>1370</v>
+        <v>243</v>
       </c>
       <c r="J13" t="n">
         <v>359</v>
@@ -1445,19 +1624,19 @@
         <v>1160</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" t="n">
         <v>468</v>
       </c>
       <c r="I14" t="n">
-        <v>2382</v>
+        <v>329</v>
       </c>
       <c r="J14" t="n">
         <v>628</v>
@@ -1476,28 +1655,28 @@
         <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1513,22 +1692,22 @@
         <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="J16" t="n">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1562,17 +1741,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1596,68 +1775,51 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Movilidad</t>
+          <t>Entorno Urbano</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PENDIENTE — sin datos cargados</t>
+          <t>PENDIENTE — por integrar</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Siniestros viales: fuente no disponible aún para la zona.</t>
+          <t>NDVI + censo arbóreo + vivienda (SISBÉN cargado, por integrar).</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Entorno Urbano</t>
+          <t>Desarrollo Económico</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PENDIENTE — sin datos cargados</t>
+          <t>PENDIENTE — por integrar</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>NDVI + censo arbóreo + vivienda: fuentes no disponibles aún.</t>
+          <t>Registro mercantil (Cámara de Comercio cargado, por integrar).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Desarrollo Económico</t>
+          <t>Educación</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PENDIENTE — sin datos cargados</t>
+          <t>PENDIENTE — por integrar</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Registro mercantil (Cámara de Comercio): no disponible aún.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Educación</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>PENDIENTE — sin datos cargados</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SIMAT/SIMPADE: no disponible aún para los colegios de la zona.</t>
+          <t>SIMAT/SIMPADE (Educacion_2026 cargado, por integrar).</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1745,7 +1907,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Seguridad (homicidios, hurtos) + Cohesión (VIF, riñas, SPA)</t>
+          <t>Seguridad + Movilidad + Cohesión (2026 integrado y anualizado)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pulmon de Oriente: 5 dimensiones completas (DE + Educacion + Entorno Urbano)
- Desarrollo Economico: Camara oficial filtrada al poligono (2387 negocios, establecimientos+empleo)
  consolidado registro_mercantil_PO_consolidado.json; build_de_pulmon_oriente.py
- Educacion: 10 colegios del poligono (spatial join sedes) -> educacion_PO_consolidado.json;
  build_educacion_pulmon_oriente.py. Entra a DesSocial (matricula+desercion)
- Entorno Urbano: NDVI real (4 tif) + habitabilidad (SISBEN sjoin+prorrateo). Censo arboreo PENDIENTE
  (el cargado era de Barrio Obrero). sec_vivienda = repo oficial del shapefile SISBEN
- ITT final 5 dim: 2023=49.8, 2024=57.4, 2025=55.6, 2026=46.0. Excel 10 hojas
- NO toca 04_itt_pulmon_oriente_2026.ipynb (base del usuario)
</commit_message>
<xml_diff>
--- a/outputs/itt_pulmon_oriente/ITT_Pulmon_Oriente_Consolidado.xlsx
+++ b/outputs/itt_pulmon_oriente/ITT_Pulmon_Oriente_Consolidado.xlsx
@@ -11,9 +11,12 @@
     <sheet name="Seguridad" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Movilidad" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cohesion_Social" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Indicadores_Trimestrales" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Dimensiones_Pendientes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Metadatos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Educacion" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Entorno_Urbano" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Desarrollo_Economico" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Indicadores_Trimestrales" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Dimensiones_Pendientes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Metadatos" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -503,12 +506,16 @@
         <v>34.21</v>
       </c>
       <c r="D2" t="n">
-        <v>75.14</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+        <v>71.63</v>
+      </c>
+      <c r="E2" t="n">
+        <v>46.28</v>
+      </c>
+      <c r="F2" t="n">
+        <v>66.7</v>
+      </c>
       <c r="G2" t="n">
-        <v>47.9</v>
+        <v>49.8</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -532,12 +539,16 @@
         <v>46.85</v>
       </c>
       <c r="D3" t="n">
-        <v>73.98999999999999</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
+        <v>65.23</v>
+      </c>
+      <c r="E3" t="n">
+        <v>52.54</v>
+      </c>
+      <c r="F3" t="n">
+        <v>76.79000000000001</v>
+      </c>
       <c r="G3" t="n">
-        <v>56.8</v>
+        <v>57.4</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -561,12 +572,16 @@
         <v>33.62</v>
       </c>
       <c r="D4" t="n">
-        <v>46.52</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
+        <v>39.64</v>
+      </c>
+      <c r="E4" t="n">
+        <v>64.94</v>
+      </c>
+      <c r="F4" t="n">
+        <v>86.95999999999999</v>
+      </c>
       <c r="G4" t="n">
-        <v>48.3</v>
+        <v>55.6</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -590,21 +605,137 @@
         <v>37.38</v>
       </c>
       <c r="D5" t="n">
-        <v>13.94</v>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
+        <v>35.45</v>
+      </c>
+      <c r="E5" t="n">
+        <v>63.77</v>
+      </c>
+      <c r="F5" t="n">
+        <v>86.95999999999999</v>
+      </c>
       <c r="G5" t="n">
-        <v>26.6</v>
+        <v>46</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Activacion</t>
+          <t>Consolidacion</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>2026 datos a la fecha (DATIC hasta Q1) — guía</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>campo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>valor</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pulmón de Oriente</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Comunas</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>13-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Área aproximada (ha)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>568.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Periodo</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2023-2026 (2026 parcial)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Fuentes con datos</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Seguridad, Movilidad, Cohesión, Educación, Desarrollo Económico, Entorno Urbano (NDVI+vivienda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Nota polígono</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Aproximado (envolvente de los eventos); polígono oficial pendiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Nota VIF</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Filtrado por los 33 barrios de la zona (no recortado espacialmente).</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1132,7 @@
         <v>66</v>
       </c>
       <c r="H2" t="n">
-        <v>75.14</v>
+        <v>71.63</v>
       </c>
     </row>
     <row r="3">
@@ -1027,7 +1158,7 @@
         <v>76.22</v>
       </c>
       <c r="H3" t="n">
-        <v>73.98999999999999</v>
+        <v>65.23</v>
       </c>
     </row>
     <row r="4">
@@ -1053,7 +1184,7 @@
         <v>39.26</v>
       </c>
       <c r="H4" t="n">
-        <v>46.52</v>
+        <v>39.64</v>
       </c>
     </row>
     <row r="5">
@@ -1079,7 +1210,7 @@
         <v>12.96</v>
       </c>
       <c r="H5" t="n">
-        <v>13.94</v>
+        <v>35.45</v>
       </c>
     </row>
   </sheetData>
@@ -1088,6 +1219,492 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>año</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>matricula</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>desertores</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>repitentes</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tasa_desercion</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tasa_repitencia</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>score_matricula</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>score_desercion</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>score_educ_des</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B2" t="n">
+        <v>18175</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1501</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2173</v>
+      </c>
+      <c r="E2" t="n">
+        <v>8.26</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11.96</v>
+      </c>
+      <c r="G2" t="n">
+        <v>87.81</v>
+      </c>
+      <c r="H2" t="n">
+        <v>44.93</v>
+      </c>
+      <c r="I2" t="n">
+        <v>42.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="n">
+        <v>17643</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1153</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2152</v>
+      </c>
+      <c r="E3" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>47.78</v>
+      </c>
+      <c r="H3" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="I3" t="n">
+        <v>47.7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" t="n">
+        <v>17008</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1054</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1820</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>58.67</v>
+      </c>
+      <c r="I4" t="n">
+        <v>52.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="n">
+        <v>18337</v>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>2009</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="G5" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>45.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>año</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>ndvi</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>arbolado</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>score_ndvi</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>score_arbolado</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>score_habitabilidad</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>score_entorno_u</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.1808</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>31.3563</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>46.2781</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>NDVI anual (satelital) + habitabilidad (1 - déficit habitacional 2024). Censo arbóreo de Pulmón PENDIENTE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.1886</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>43.8807</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>52.5404</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>NDVI anual (satelital) + habitabilidad (1 - déficit habitacional 2024). Censo arbóreo de Pulmón PENDIENTE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.2043</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>68.6832</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>64.94159999999999</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>NDVI anual (satelital) + habitabilidad (1 - déficit habitacional 2024). Censo arbóreo de Pulmón PENDIENTE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.2028</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>66.3442</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>61.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>63.7721</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>NDVI anual (satelital) + habitabilidad (1 - déficit habitacional 2024). Censo arbóreo de Pulmón PENDIENTE.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>año</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>establecimientos_activos</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>empleo_personas</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>score_establecimientos</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>score_empleo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>score_des_eco</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1543</v>
+      </c>
+      <c r="C2" t="n">
+        <v>2393</v>
+      </c>
+      <c r="D2" t="n">
+        <v>56.21</v>
+      </c>
+      <c r="E2" t="n">
+        <v>77.18000000000001</v>
+      </c>
+      <c r="F2" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1942</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2568</v>
+      </c>
+      <c r="D3" t="n">
+        <v>70.75</v>
+      </c>
+      <c r="E3" t="n">
+        <v>82.83</v>
+      </c>
+      <c r="F3" t="n">
+        <v>76.79000000000001</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B4" t="n">
+        <v>2387</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2696</v>
+      </c>
+      <c r="D4" t="n">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="E4" t="n">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="F4" t="n">
+        <v>86.95999999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2387</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2696</v>
+      </c>
+      <c r="D5" t="n">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="E5" t="n">
+        <v>86.95999999999999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>86.95999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1741,17 +2358,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1775,163 +2392,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Entorno Urbano</t>
+          <t>Censo arbóreo (Entorno Urbano)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PENDIENTE — por integrar</t>
+          <t>PENDIENTE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>NDVI + censo arbóreo + vivienda (SISBÉN cargado, por integrar).</t>
+          <t>El censo arbóreo cargado era de Barrio Obrero; falta el de Pulmón. EntornoU usa NDVI + habitabilidad.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Desarrollo Económico</t>
+          <t>Polígono oficial</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PENDIENTE — por integrar</t>
+          <t>PENDIENTE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Registro mercantil (Cámara de Comercio cargado, por integrar).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Educación</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>PENDIENTE — por integrar</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>SIMAT/SIMPADE (Educacion_2026 cargado, por integrar).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>campo</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>valor</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Zona</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Pulmón de Oriente</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Comunas</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>13-14</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Área aproximada (ha)</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>568.4</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Periodo</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2023-2026 (2026 parcial)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Fuentes con datos</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Seguridad + Movilidad + Cohesión (2026 integrado y anualizado)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Nota polígono</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Aproximado (envolvente de los eventos); polígono oficial pendiente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Nota VIF</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Filtrado por los 33 barrios de la zona (no recortado espacialmente).</t>
+          <t>Polígono aproximado (envolvente de eventos ~568 ha); falta el oficial.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Pulmon de Oriente: integra censo arboreo real al Entorno Urbano
- Censo real CENSO_ARBOREO_poligono_Oriente.geojson (20459 arboles dentro
  del poligono, 20196 vivos/nuevos) reemplaza el censo erroneo de Barrio Obrero.
- score_arbolado ahora se calcula (umbral 0-30294); score_entorno_u pasa a
  3 componentes reales (NDVI + arbolado + habitabilidad).
- EntornoU: 53.1/57.2/65.5/64.7 (antes 46.3/52.5/64.9/63.8).
- ITT 5-dim: 2023=51.0, 2024=58.2, 2025=55.7, 2026=46.2 (Consolidacion).
- Dimensiones_Pendientes queda solo con poligono oficial; Excel regenerado.
</commit_message>
<xml_diff>
--- a/outputs/itt_pulmon_oriente/ITT_Pulmon_Oriente_Consolidado.xlsx
+++ b/outputs/itt_pulmon_oriente/ITT_Pulmon_Oriente_Consolidado.xlsx
@@ -509,13 +509,13 @@
         <v>71.63</v>
       </c>
       <c r="E2" t="n">
-        <v>46.28</v>
+        <v>53.07</v>
       </c>
       <c r="F2" t="n">
         <v>66.7</v>
       </c>
       <c r="G2" t="n">
-        <v>49.8</v>
+        <v>51</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -542,13 +542,13 @@
         <v>65.23</v>
       </c>
       <c r="E3" t="n">
-        <v>52.54</v>
+        <v>57.25</v>
       </c>
       <c r="F3" t="n">
         <v>76.79000000000001</v>
       </c>
       <c r="G3" t="n">
-        <v>57.4</v>
+        <v>58.2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -575,13 +575,13 @@
         <v>39.64</v>
       </c>
       <c r="E4" t="n">
-        <v>64.94</v>
+        <v>65.52</v>
       </c>
       <c r="F4" t="n">
         <v>86.95999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>55.6</v>
+        <v>55.7</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -608,13 +608,13 @@
         <v>35.45</v>
       </c>
       <c r="E5" t="n">
-        <v>63.77</v>
+        <v>64.73999999999999</v>
       </c>
       <c r="F5" t="n">
         <v>86.95999999999999</v>
       </c>
       <c r="G5" t="n">
-        <v>46</v>
+        <v>46.2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1469,21 +1469,23 @@
         <v>0.1808</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>20196</v>
       </c>
       <c r="D2" t="n">
         <v>31.3563</v>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>66.66670000000001</v>
+      </c>
       <c r="F2" t="n">
         <v>61.2</v>
       </c>
       <c r="G2" t="n">
-        <v>46.2781</v>
+        <v>53.0743</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>NDVI anual (satelital) + habitabilidad (1 - déficit habitacional 2024). Censo arbóreo de Pulmón PENDIENTE.</t>
+          <t>NDVI anual (satelital) + censo arbóreo real (árboles vivos/nuevos dentro del polígono) + habitabilidad (1 - déficit habitacional 2024).</t>
         </is>
       </c>
     </row>
@@ -1495,21 +1497,23 @@
         <v>0.1886</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>20196</v>
       </c>
       <c r="D3" t="n">
         <v>43.8807</v>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>66.66670000000001</v>
+      </c>
       <c r="F3" t="n">
         <v>61.2</v>
       </c>
       <c r="G3" t="n">
-        <v>52.5404</v>
+        <v>57.2491</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>NDVI anual (satelital) + habitabilidad (1 - déficit habitacional 2024). Censo arbóreo de Pulmón PENDIENTE.</t>
+          <t>NDVI anual (satelital) + censo arbóreo real (árboles vivos/nuevos dentro del polígono) + habitabilidad (1 - déficit habitacional 2024).</t>
         </is>
       </c>
     </row>
@@ -1521,21 +1525,23 @@
         <v>0.2043</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>20196</v>
       </c>
       <c r="D4" t="n">
         <v>68.6832</v>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>66.66670000000001</v>
+      </c>
       <c r="F4" t="n">
         <v>61.2</v>
       </c>
       <c r="G4" t="n">
-        <v>64.94159999999999</v>
+        <v>65.5166</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NDVI anual (satelital) + habitabilidad (1 - déficit habitacional 2024). Censo arbóreo de Pulmón PENDIENTE.</t>
+          <t>NDVI anual (satelital) + censo arbóreo real (árboles vivos/nuevos dentro del polígono) + habitabilidad (1 - déficit habitacional 2024).</t>
         </is>
       </c>
     </row>
@@ -1547,21 +1553,23 @@
         <v>0.2028</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>20196</v>
       </c>
       <c r="D5" t="n">
         <v>66.3442</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>66.66670000000001</v>
+      </c>
       <c r="F5" t="n">
         <v>61.2</v>
       </c>
       <c r="G5" t="n">
-        <v>63.7721</v>
+        <v>64.73699999999999</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NDVI anual (satelital) + habitabilidad (1 - déficit habitacional 2024). Censo arbóreo de Pulmón PENDIENTE.</t>
+          <t>NDVI anual (satelital) + censo arbóreo real (árboles vivos/nuevos dentro del polígono) + habitabilidad (1 - déficit habitacional 2024).</t>
         </is>
       </c>
     </row>
@@ -2364,10 +2372,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
@@ -2392,7 +2400,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Censo arbóreo (Entorno Urbano)</t>
+          <t>Polígono oficial</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2402,24 +2410,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>El censo arbóreo cargado era de Barrio Obrero; falta el de Pulmón. EntornoU usa NDVI + habitabilidad.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Polígono oficial</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Polígono aproximado (envolvente de eventos ~568 ha); falta el oficial.</t>
+          <t>Polígono aproximado (envolvente de eventos ~568 ha); falta el oficial de planeación.</t>
         </is>
       </c>
     </row>

</xml_diff>